<commit_message>
docs: continue work on calibration functions; delete some unnecessary stuff
</commit_message>
<xml_diff>
--- a/docs/spectra/calibration_function.xlsx
+++ b/docs/spectra/calibration_function.xlsx
@@ -8,12 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andre\Documents\Schule\Unterricht\Informatik\repos\vernier-cs\docs\spectra\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0302AD97-D31F-4EBD-AABA-5FE1DB16AA2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D410FFD-3F6C-41EC-8504-D79D71372BD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="20777" windowHeight="13200" xr2:uid="{B0D95946-56EA-4653-A34B-847126CFC8AD}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="20777" windowHeight="13200" activeTab="2" xr2:uid="{B0D95946-56EA-4653-A34B-847126CFC8AD}"/>
   </bookViews>
   <sheets>
     <sheet name="SpectroVisPlus" sheetId="1" r:id="rId1"/>
+    <sheet name="SpectroVis" sheetId="2" r:id="rId2"/>
+    <sheet name="SpectroVisPlusBLE" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="2">
   <si>
     <t>λ [nm]</t>
   </si>
@@ -2014,25 +2016,25 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="578"/>
                 <c:pt idx="114">
-                  <c:v>713</c:v>
+                  <c:v>712</c:v>
                 </c:pt>
                 <c:pt idx="177">
-                  <c:v>781</c:v>
+                  <c:v>780</c:v>
                 </c:pt>
                 <c:pt idx="228">
-                  <c:v>834</c:v>
+                  <c:v>833</c:v>
                 </c:pt>
                 <c:pt idx="229">
-                  <c:v>837</c:v>
+                  <c:v>836</c:v>
                 </c:pt>
                 <c:pt idx="255">
-                  <c:v>868</c:v>
+                  <c:v>867</c:v>
                 </c:pt>
                 <c:pt idx="319">
-                  <c:v>945</c:v>
+                  <c:v>944</c:v>
                 </c:pt>
                 <c:pt idx="364">
-                  <c:v>998</c:v>
+                  <c:v>997</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2343,7 +2345,807 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="de-DE"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Kalibrierfunktion SpectroVis</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="de-DE"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>SpectroVis!$B$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Pixelindex</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="38100" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="linear"/>
+            <c:dispRSqr val="1"/>
+            <c:dispEq val="1"/>
+            <c:trendlineLbl>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-0.16648490813648295"/>
+                  <c:y val="-5.0462962962962961E-3"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:numFmt formatCode="General" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="65000"/>
+                          <a:lumOff val="35000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="de-DE"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
+          </c:trendline>
+          <c:xVal>
+            <c:numRef>
+              <c:f>SpectroVis!$A$2:$A$87</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="86"/>
+                <c:pt idx="0">
+                  <c:v>403.25</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>407</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>410.75</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>414.5</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>418.25</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>422</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>425.75</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>429.5</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>433.25</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>437</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>440.75</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>444.5</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>448.25</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>452</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>455.75</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>459.5</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>463.25</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>467</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>470.75</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>474.5</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>478.25</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>482</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>485.75</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>489.5</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>493.25</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>497</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>500.75</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>504.5</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>508.25</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>512</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>515.75</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>519.5</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>523.25</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>527</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>530.75</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>534.5</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>538.25</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>542</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>545.27</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>549.5</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>553.25</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>557</c:v>
+                </c:pt>
+                <c:pt idx="42">
+                  <c:v>560.75</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>564.5</c:v>
+                </c:pt>
+                <c:pt idx="44">
+                  <c:v>568.25</c:v>
+                </c:pt>
+                <c:pt idx="45">
+                  <c:v>572</c:v>
+                </c:pt>
+                <c:pt idx="46">
+                  <c:v>575.75</c:v>
+                </c:pt>
+                <c:pt idx="47">
+                  <c:v>579.5</c:v>
+                </c:pt>
+                <c:pt idx="48">
+                  <c:v>585.05999999999995</c:v>
+                </c:pt>
+                <c:pt idx="49">
+                  <c:v>587</c:v>
+                </c:pt>
+                <c:pt idx="50">
+                  <c:v>590.75</c:v>
+                </c:pt>
+                <c:pt idx="51">
+                  <c:v>594.5</c:v>
+                </c:pt>
+                <c:pt idx="52">
+                  <c:v>598.25</c:v>
+                </c:pt>
+                <c:pt idx="53">
+                  <c:v>602</c:v>
+                </c:pt>
+                <c:pt idx="54">
+                  <c:v>605.75</c:v>
+                </c:pt>
+                <c:pt idx="55">
+                  <c:v>609.5</c:v>
+                </c:pt>
+                <c:pt idx="56">
+                  <c:v>611.67999999999995</c:v>
+                </c:pt>
+                <c:pt idx="57">
+                  <c:v>617</c:v>
+                </c:pt>
+                <c:pt idx="58">
+                  <c:v>620.75</c:v>
+                </c:pt>
+                <c:pt idx="59">
+                  <c:v>624.5</c:v>
+                </c:pt>
+                <c:pt idx="60">
+                  <c:v>628.25</c:v>
+                </c:pt>
+                <c:pt idx="61">
+                  <c:v>632</c:v>
+                </c:pt>
+                <c:pt idx="62">
+                  <c:v>635.75</c:v>
+                </c:pt>
+                <c:pt idx="63">
+                  <c:v>639.5</c:v>
+                </c:pt>
+                <c:pt idx="64">
+                  <c:v>643.25</c:v>
+                </c:pt>
+                <c:pt idx="65">
+                  <c:v>647</c:v>
+                </c:pt>
+                <c:pt idx="66">
+                  <c:v>650.75</c:v>
+                </c:pt>
+                <c:pt idx="67">
+                  <c:v>654.5</c:v>
+                </c:pt>
+                <c:pt idx="68">
+                  <c:v>658.25</c:v>
+                </c:pt>
+                <c:pt idx="69">
+                  <c:v>662</c:v>
+                </c:pt>
+                <c:pt idx="70">
+                  <c:v>665.75</c:v>
+                </c:pt>
+                <c:pt idx="71">
+                  <c:v>669.5</c:v>
+                </c:pt>
+                <c:pt idx="72">
+                  <c:v>673.25</c:v>
+                </c:pt>
+                <c:pt idx="73">
+                  <c:v>677</c:v>
+                </c:pt>
+                <c:pt idx="74">
+                  <c:v>680.75</c:v>
+                </c:pt>
+                <c:pt idx="75">
+                  <c:v>684.5</c:v>
+                </c:pt>
+                <c:pt idx="76">
+                  <c:v>688.25</c:v>
+                </c:pt>
+                <c:pt idx="77">
+                  <c:v>692</c:v>
+                </c:pt>
+                <c:pt idx="78">
+                  <c:v>695.75</c:v>
+                </c:pt>
+                <c:pt idx="79">
+                  <c:v>698</c:v>
+                </c:pt>
+                <c:pt idx="80">
+                  <c:v>703.25</c:v>
+                </c:pt>
+                <c:pt idx="81">
+                  <c:v>707</c:v>
+                </c:pt>
+                <c:pt idx="82">
+                  <c:v>710.75</c:v>
+                </c:pt>
+                <c:pt idx="83">
+                  <c:v>714.5</c:v>
+                </c:pt>
+                <c:pt idx="84">
+                  <c:v>718.25</c:v>
+                </c:pt>
+                <c:pt idx="85">
+                  <c:v>722</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>SpectroVis!$B$2:$B$87</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="86"/>
+                <c:pt idx="23">
+                  <c:v>86</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>104</c:v>
+                </c:pt>
+                <c:pt idx="48">
+                  <c:v>118</c:v>
+                </c:pt>
+                <c:pt idx="56">
+                  <c:v>126</c:v>
+                </c:pt>
+                <c:pt idx="79">
+                  <c:v>152</c:v>
+                </c:pt>
+                <c:pt idx="81">
+                  <c:v>158</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-3EA0-4FEE-9699-D01E35B2B0EF}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="1648324799"/>
+        <c:axId val="1648326239"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="1648324799"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:min val="400"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="de-CH"/>
+                  <a:t>Wellenlänge [nm]</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="de-DE"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="de-DE"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1648326239"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="1648326239"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="de-CH"/>
+                  <a:t>Pixelindex</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="de-DE"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="de-DE"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1648324799"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="de-DE"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.78740157499999996" l="0.7" r="0.7" t="0.78740157499999996" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
   <a:schemeClr val="accent2"/>
@@ -2899,20 +3701,536 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>228599</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>81642</xdr:rowOff>
+      <xdr:colOff>821871</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>21771</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>664028</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>48985</xdr:rowOff>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>429986</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>174171</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -2920,6 +4238,47 @@
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{580BA637-05AB-C705-0107-59C0A21DDCEC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>402770</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>157842</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>10885</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>125185</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Diagramm 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{43E941CE-B435-139B-49EE-07651EAB209E}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3843,7 +5202,7 @@
         <v>483.3</v>
       </c>
       <c r="B116">
-        <v>713</v>
+        <v>712</v>
       </c>
     </row>
     <row r="117" spans="1:2" x14ac:dyDescent="0.4">
@@ -4161,7 +5520,7 @@
         <v>539.899999999996</v>
       </c>
       <c r="B179">
-        <v>781</v>
+        <v>780</v>
       </c>
     </row>
     <row r="180" spans="1:2" x14ac:dyDescent="0.4">
@@ -4419,7 +5778,7 @@
         <v>585.70000000000005</v>
       </c>
       <c r="B230">
-        <v>834</v>
+        <v>833</v>
       </c>
     </row>
     <row r="231" spans="1:2" x14ac:dyDescent="0.4">
@@ -4427,7 +5786,7 @@
         <v>586.5</v>
       </c>
       <c r="B231">
-        <v>837</v>
+        <v>836</v>
       </c>
     </row>
     <row r="232" spans="1:2" x14ac:dyDescent="0.4">
@@ -4560,7 +5919,7 @@
         <v>610.6</v>
       </c>
       <c r="B257">
-        <v>868</v>
+        <v>867</v>
       </c>
     </row>
     <row r="258" spans="1:2" x14ac:dyDescent="0.4">
@@ -4883,7 +6242,7 @@
         <v>667.4</v>
       </c>
       <c r="B321">
-        <v>945</v>
+        <v>944</v>
       </c>
     </row>
     <row r="322" spans="1:2" x14ac:dyDescent="0.4">
@@ -5111,7 +6470,7 @@
         <v>708.3</v>
       </c>
       <c r="B366">
-        <v>998</v>
+        <v>997</v>
       </c>
     </row>
     <row r="367" spans="1:2" x14ac:dyDescent="0.4">
@@ -6183,4 +7542,489 @@
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B682566-8A20-49A7-A371-C42E121E5F1C}">
+  <dimension ref="A1:B87"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A2">
+        <v>403.25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A3">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A4">
+        <v>410.75</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A5">
+        <v>414.5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A6">
+        <v>418.25</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A7">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A8">
+        <v>425.75</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A9">
+        <v>429.5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A10">
+        <v>433.25</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A11">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A12">
+        <v>440.75</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A13">
+        <v>444.5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A14">
+        <v>448.25</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A15">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A16">
+        <v>455.75</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A17">
+        <v>459.5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A18">
+        <v>463.25</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A19">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A20">
+        <v>470.75</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A21">
+        <v>474.5</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A22">
+        <v>478.25</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A23">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A24">
+        <v>485.75</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A25">
+        <v>489.5</v>
+      </c>
+      <c r="B25">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A26">
+        <v>493.25</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A27">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A28">
+        <v>500.75</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A29">
+        <v>504.5</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A30">
+        <v>508.25</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A31">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A32">
+        <v>515.75</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A33">
+        <v>519.5</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A34">
+        <v>523.25</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A35">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A36">
+        <v>530.75</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A37">
+        <v>534.5</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A38">
+        <v>538.25</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A39">
+        <v>542</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A40">
+        <v>545.27</v>
+      </c>
+      <c r="B40">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A41">
+        <v>549.5</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A42">
+        <v>553.25</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A43">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A44">
+        <v>560.75</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A45">
+        <v>564.5</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A46">
+        <v>568.25</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A47">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A48">
+        <v>575.75</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A49">
+        <v>579.5</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A50">
+        <v>585.05999999999995</v>
+      </c>
+      <c r="B50">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A51">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A52">
+        <v>590.75</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A53">
+        <v>594.5</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A54">
+        <v>598.25</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A55">
+        <v>602</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A56">
+        <v>605.75</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A57">
+        <v>609.5</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A58">
+        <v>611.67999999999995</v>
+      </c>
+      <c r="B58">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A59">
+        <v>617</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A60">
+        <v>620.75</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A61">
+        <v>624.5</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A62">
+        <v>628.25</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A63">
+        <v>632</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A64">
+        <v>635.75</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A65">
+        <v>639.5</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A66">
+        <v>643.25</v>
+      </c>
+    </row>
+    <row r="67" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A67">
+        <v>647</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A68">
+        <v>650.75</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A69">
+        <v>654.5</v>
+      </c>
+    </row>
+    <row r="70" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A70">
+        <v>658.25</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A71">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A72">
+        <v>665.75</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A73">
+        <v>669.5</v>
+      </c>
+    </row>
+    <row r="74" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A74">
+        <v>673.25</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A75">
+        <v>677</v>
+      </c>
+    </row>
+    <row r="76" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A76">
+        <v>680.75</v>
+      </c>
+    </row>
+    <row r="77" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A77">
+        <v>684.5</v>
+      </c>
+    </row>
+    <row r="78" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A78">
+        <v>688.25</v>
+      </c>
+    </row>
+    <row r="79" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A79">
+        <v>692</v>
+      </c>
+    </row>
+    <row r="80" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A80">
+        <v>695.75</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A81">
+        <v>698</v>
+      </c>
+      <c r="B81">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A82">
+        <v>703.25</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A83">
+        <v>707</v>
+      </c>
+      <c r="B83">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A84">
+        <v>710.75</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A85">
+        <v>714.5</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A86">
+        <v>718.25</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A87">
+        <v>722</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4AAC00CE-4EE9-46E8-A686-2D14982E558B}">
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>